<commit_message>
made progress in the database
</commit_message>
<xml_diff>
--- a/dist/master_workbook.xlsx
+++ b/dist/master_workbook.xlsx
@@ -8,17 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carcheme\PycharmProjects\request_template\dist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64789A8F-0BD7-4B1A-9233-36935CBCF580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D36558E-2CEE-446B-BA70-EBFAFB4D0E21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1830" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="digestion_page" sheetId="1" r:id="rId1"/>
-    <sheet name="200128035" sheetId="2" r:id="rId2"/>
-    <sheet name="200128036" sheetId="3" r:id="rId3"/>
-    <sheet name="200128037" sheetId="4" r:id="rId4"/>
-    <sheet name="200128038" sheetId="5" r:id="rId5"/>
-    <sheet name="formula_page" sheetId="6" r:id="rId6"/>
+    <sheet name="200128032" sheetId="2" r:id="rId2"/>
+    <sheet name="200128033" sheetId="3" r:id="rId3"/>
+    <sheet name="200128034" sheetId="4" r:id="rId4"/>
+    <sheet name="formula_page" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="49">
   <si>
     <t>Date:</t>
   </si>
@@ -46,7 +45,7 @@
     <t>Request ID:</t>
   </si>
   <si>
-    <t>100048569</t>
+    <t>100048568</t>
   </si>
   <si>
     <t>Microwave</t>
@@ -55,7 +54,7 @@
     <t>Element(s)</t>
   </si>
   <si>
-    <t>Cu</t>
+    <t>Ca</t>
   </si>
   <si>
     <t>SOP#</t>
@@ -97,31 +96,25 @@
     <t>volume (mL)</t>
   </si>
   <si>
-    <t>200128035_1</t>
-  </si>
-  <si>
-    <t>200128035_2</t>
-  </si>
-  <si>
-    <t>200128036_1</t>
-  </si>
-  <si>
-    <t>200128036_2</t>
-  </si>
-  <si>
-    <t>200128037_1</t>
-  </si>
-  <si>
-    <t>200128037_2</t>
-  </si>
-  <si>
-    <t>200128038_1</t>
-  </si>
-  <si>
-    <t>200128038_2</t>
-  </si>
-  <si>
-    <t>Cu ICP analysis</t>
+    <t>200128032_1</t>
+  </si>
+  <si>
+    <t>200128032_2</t>
+  </si>
+  <si>
+    <t>200128033_1</t>
+  </si>
+  <si>
+    <t>200128033_2</t>
+  </si>
+  <si>
+    <t>200128034_1</t>
+  </si>
+  <si>
+    <t>200128034_2</t>
+  </si>
+  <si>
+    <t>Ca ICP analysis</t>
   </si>
   <si>
     <t>sample</t>
@@ -133,22 +126,22 @@
     <t>conc. [mg/L]</t>
   </si>
   <si>
-    <t>Cu_ppm</t>
-  </si>
-  <si>
-    <t>%Cu</t>
-  </si>
-  <si>
-    <t>cu result:</t>
-  </si>
-  <si>
-    <t>cu oxide factor:</t>
-  </si>
-  <si>
-    <t>cu oxide result:</t>
-  </si>
-  <si>
-    <t>cu lot:</t>
+    <t>Ca_ppm</t>
+  </si>
+  <si>
+    <t>%Ca</t>
+  </si>
+  <si>
+    <t>ca result:</t>
+  </si>
+  <si>
+    <t>ca oxide factor:</t>
+  </si>
+  <si>
+    <t>ca oxide result:</t>
+  </si>
+  <si>
+    <t>ca lot:</t>
   </si>
   <si>
     <t>Note(s):</t>
@@ -191,12 +184,6 @@
   </si>
   <si>
     <t>%Cr(III) = total_Cr - Cr(VI)</t>
-  </si>
-  <si>
-    <t>Quartz</t>
-  </si>
-  <si>
-    <t>3 mL HCl, 1 mL HNO3</t>
   </si>
 </sst>
 </file>
@@ -251,12 +238,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -286,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -330,21 +323,17 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill>
@@ -666,7 +655,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -681,7 +670,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -725,9 +714,7 @@
       <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>52</v>
-      </c>
+      <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
@@ -736,9 +723,7 @@
       <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="16">
-        <v>20</v>
-      </c>
+      <c r="B9" s="16"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
@@ -747,9 +732,7 @@
       <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="15" t="s">
-        <v>51</v>
-      </c>
+      <c r="B10" s="15"/>
       <c r="C10" s="15"/>
       <c r="D10" s="15"/>
       <c r="E10" s="15"/>
@@ -758,9 +741,7 @@
       <c r="A11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="21">
-        <v>0</v>
-      </c>
+      <c r="B11" s="16"/>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
@@ -817,21 +798,11 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="5">
-        <v>30</v>
-      </c>
-      <c r="B15" s="5">
-        <v>1500</v>
-      </c>
-      <c r="C15" s="5">
-        <v>240</v>
-      </c>
-      <c r="D15" s="5">
-        <v>65</v>
-      </c>
-      <c r="E15" s="5">
-        <v>110</v>
-      </c>
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
@@ -848,7 +819,9 @@
       <c r="A17" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="6"/>
+      <c r="B17" s="6">
+        <v>0.30559999999999998</v>
+      </c>
       <c r="C17" s="5">
         <v>250</v>
       </c>
@@ -857,7 +830,9 @@
       <c r="A18" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="6"/>
+      <c r="B18" s="6">
+        <v>0.30170000000000002</v>
+      </c>
       <c r="C18" s="5">
         <v>250</v>
       </c>
@@ -866,7 +841,9 @@
       <c r="A19" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="6"/>
+      <c r="B19" s="6">
+        <v>0.30359999999999998</v>
+      </c>
       <c r="C19" s="5">
         <v>250</v>
       </c>
@@ -875,7 +852,9 @@
       <c r="A20" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="6"/>
+      <c r="B20" s="6">
+        <v>0.30230000000000001</v>
+      </c>
       <c r="C20" s="5">
         <v>250</v>
       </c>
@@ -884,7 +863,9 @@
       <c r="A21" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="6"/>
+      <c r="B21" s="6">
+        <v>0.30690000000000001</v>
+      </c>
       <c r="C21" s="5">
         <v>250</v>
       </c>
@@ -893,26 +874,10 @@
       <c r="A22" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="6"/>
+      <c r="B22" s="6">
+        <v>0.30570000000000003</v>
+      </c>
       <c r="C22" s="5">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23" s="6"/>
-      <c r="C23" s="5">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="5">
         <v>250</v>
       </c>
     </row>
@@ -935,11 +900,11 @@
   <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -947,7 +912,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -960,25 +925,25 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B5" s="17"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -986,21 +951,23 @@
         <v>19</v>
       </c>
       <c r="B7" s="5" t="str">
-        <f>"1/1"</f>
-        <v>1/1</v>
-      </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="8" t="e">
+        <f>"50/1"</f>
+        <v>50/1</v>
+      </c>
+      <c r="C7" s="7">
+        <v>1.1575</v>
+      </c>
+      <c r="D7" s="8">
         <f>((C7)*(H7)*(I7))/(G7*1)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E7" s="8" t="e">
+        <v>47345.386125654455</v>
+      </c>
+      <c r="E7" s="8">
         <f>D7/10000</f>
-        <v>#DIV/0!</v>
+        <v>4.7345386125654452</v>
       </c>
       <c r="G7" s="9">
         <f>digestion_page!B17</f>
-        <v>0</v>
+        <v>0.30559999999999998</v>
       </c>
       <c r="H7" s="9">
         <f>digestion_page!C17</f>
@@ -1008,7 +975,7 @@
       </c>
       <c r="I7" s="9">
         <f>(LEFT(B7,FIND("/",B7)-1)/RIGHT(B7,LEN(B7)-FIND("/", B7)))</f>
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1016,21 +983,23 @@
         <v>20</v>
       </c>
       <c r="B8" s="5" t="str">
-        <f>"1/1"</f>
-        <v>1/1</v>
-      </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="8" t="e">
+        <f>"50/1"</f>
+        <v>50/1</v>
+      </c>
+      <c r="C8" s="7">
+        <v>1.2275</v>
+      </c>
+      <c r="D8" s="8">
         <f>((C8)*(H8)*(I8))/(G8*1)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E8" s="8" t="e">
+        <v>50857.640039774604</v>
+      </c>
+      <c r="E8" s="8">
         <f>D8/10000</f>
-        <v>#DIV/0!</v>
+        <v>5.0857640039774603</v>
       </c>
       <c r="G8" s="9">
         <f>digestion_page!B18</f>
-        <v>0</v>
+        <v>0.30170000000000002</v>
       </c>
       <c r="H8" s="9">
         <f>digestion_page!C18</f>
@@ -1038,49 +1007,51 @@
       </c>
       <c r="I8" s="9">
         <f>(LEFT(B8,FIND("/",B8)-1)/RIGHT(B8,LEN(B8)-FIND("/", B8)))</f>
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" s="18"/>
-      <c r="C10" s="11" t="e">
+      <c r="C10" s="11">
         <f>AVERAGE(D7:D8)</f>
-        <v>#DIV/0!</v>
+        <v>49101.513082714533</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B11" s="18"/>
-      <c r="C11" s="12" t="e">
+      <c r="C11" s="12">
         <f>AVERAGE(E7:E8)</f>
-        <v>#DIV/0!</v>
+        <v>4.9101513082714527</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B12" s="18"/>
-      <c r="C12" s="3"/>
+      <c r="C12" s="3">
+        <v>1.399</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="12" t="e">
+      <c r="A13" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="21"/>
+      <c r="C13" s="22">
         <f>AVERAGE(E7:E8)*(C12)</f>
-        <v>#DIV/0!</v>
+        <v>6.8693016802717626</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B14" s="18"/>
       <c r="C14" s="19"/>
@@ -1090,206 +1061,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B16" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-    </row>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-    </row>
-    <row r="18" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-    </row>
-  </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="C16:F18"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-  </mergeCells>
-  <conditionalFormatting sqref="C14:F14">
-    <cfRule type="containsBlanks" dxfId="3" priority="1">
-      <formula>LEN(TRIM(C14))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2">
-        <v>46161</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="17"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="5" t="str">
-        <f>"1/1"</f>
-        <v>1/1</v>
-      </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="8" t="e">
-        <f>((C7)*(H7)*(I7))/(G7*1)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E7" s="8" t="e">
-        <f>D7/10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G7" s="9">
-        <f>digestion_page!B19</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="9">
-        <f>digestion_page!C19</f>
-        <v>250</v>
-      </c>
-      <c r="I7" s="9">
-        <f>(LEFT(B7,FIND("/",B7)-1)/RIGHT(B7,LEN(B7)-FIND("/", B7)))</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="5" t="str">
-        <f>"1/1"</f>
-        <v>1/1</v>
-      </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="8" t="e">
-        <f>((C8)*(H8)*(I8))/(G8*1)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E8" s="8" t="e">
-        <f>D8/10000</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G8" s="9">
-        <f>digestion_page!B20</f>
-        <v>0</v>
-      </c>
-      <c r="H8" s="9">
-        <f>digestion_page!C20</f>
-        <v>250</v>
-      </c>
-      <c r="I8" s="9">
-        <f>(LEFT(B8,FIND("/",B8)-1)/RIGHT(B8,LEN(B8)-FIND("/", B8)))</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="11" t="e">
-        <f>AVERAGE(D7:D8)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="12" t="e">
-        <f>AVERAGE(E7:E8)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="3"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
         <v>35</v>
-      </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="12" t="e">
-        <f>AVERAGE(E7:E8)*(C12)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="10" t="s">
-        <v>37</v>
       </c>
       <c r="C16" s="20"/>
       <c r="D16" s="20"/>
@@ -1328,16 +1100,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1345,7 +1117,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -1358,127 +1130,133 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B5" s="17"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B7" s="5" t="str">
-        <f>"1/1"</f>
-        <v>1/1</v>
-      </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="8" t="e">
+        <f>"50/1"</f>
+        <v>50/1</v>
+      </c>
+      <c r="C7" s="7">
+        <v>2.3450000000000002</v>
+      </c>
+      <c r="D7" s="8">
         <f>((C7)*(H7)*(I7))/(G7*1)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E7" s="8" t="e">
+        <v>96549.736495388672</v>
+      </c>
+      <c r="E7" s="8">
         <f>D7/10000</f>
-        <v>#DIV/0!</v>
+        <v>9.6549736495388672</v>
       </c>
       <c r="G7" s="9">
-        <f>digestion_page!B21</f>
-        <v>0</v>
+        <f>digestion_page!B19</f>
+        <v>0.30359999999999998</v>
       </c>
       <c r="H7" s="9">
-        <f>digestion_page!C21</f>
+        <f>digestion_page!C19</f>
         <v>250</v>
       </c>
       <c r="I7" s="9">
         <f>(LEFT(B7,FIND("/",B7)-1)/RIGHT(B7,LEN(B7)-FIND("/", B7)))</f>
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B8" s="5" t="str">
-        <f>"1/1"</f>
-        <v>1/1</v>
-      </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="8" t="e">
+        <f>"50/1"</f>
+        <v>50/1</v>
+      </c>
+      <c r="C8" s="7">
+        <v>2.2725</v>
+      </c>
+      <c r="D8" s="8">
         <f>((C8)*(H8)*(I8))/(G8*1)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E8" s="8" t="e">
+        <v>93967.085676480317</v>
+      </c>
+      <c r="E8" s="8">
         <f>D8/10000</f>
-        <v>#DIV/0!</v>
+        <v>9.396708567648032</v>
       </c>
       <c r="G8" s="9">
-        <f>digestion_page!B22</f>
-        <v>0</v>
+        <f>digestion_page!B20</f>
+        <v>0.30230000000000001</v>
       </c>
       <c r="H8" s="9">
-        <f>digestion_page!C22</f>
+        <f>digestion_page!C20</f>
         <v>250</v>
       </c>
       <c r="I8" s="9">
         <f>(LEFT(B8,FIND("/",B8)-1)/RIGHT(B8,LEN(B8)-FIND("/", B8)))</f>
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" s="18"/>
-      <c r="C10" s="11" t="e">
+      <c r="C10" s="11">
         <f>AVERAGE(D7:D8)</f>
-        <v>#DIV/0!</v>
+        <v>95258.411085934495</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B11" s="18"/>
-      <c r="C11" s="12" t="e">
+      <c r="C11" s="12">
         <f>AVERAGE(E7:E8)</f>
-        <v>#DIV/0!</v>
+        <v>9.5258411085934505</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B12" s="18"/>
-      <c r="C12" s="3"/>
+      <c r="C12" s="3">
+        <v>1.399</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="12" t="e">
+      <c r="A13" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="21"/>
+      <c r="C13" s="22">
         <f>AVERAGE(E7:E8)*(C12)</f>
-        <v>#DIV/0!</v>
+        <v>13.326651710922237</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B14" s="18"/>
       <c r="C14" s="19"/>
@@ -1488,7 +1266,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B16" s="10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C16" s="20"/>
       <c r="D16" s="20"/>
@@ -1527,16 +1305,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1544,7 +1322,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>46161</v>
+        <v>46162</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -1557,127 +1335,133 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B5" s="17"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B7" s="5" t="str">
-        <f>"1/1"</f>
-        <v>1/1</v>
-      </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="8" t="e">
+        <f>"100/1"</f>
+        <v>100/1</v>
+      </c>
+      <c r="C7" s="7">
+        <v>1.69</v>
+      </c>
+      <c r="D7" s="8">
         <f>((C7)*(H7)*(I7))/(G7*1)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E7" s="8" t="e">
+        <v>137666.99250570219</v>
+      </c>
+      <c r="E7" s="8">
         <f>D7/10000</f>
-        <v>#DIV/0!</v>
+        <v>13.76669925057022</v>
       </c>
       <c r="G7" s="9">
-        <f>digestion_page!B23</f>
-        <v>0</v>
+        <f>digestion_page!B21</f>
+        <v>0.30690000000000001</v>
       </c>
       <c r="H7" s="9">
-        <f>digestion_page!C23</f>
+        <f>digestion_page!C21</f>
         <v>250</v>
       </c>
       <c r="I7" s="9">
         <f>(LEFT(B7,FIND("/",B7)-1)/RIGHT(B7,LEN(B7)-FIND("/", B7)))</f>
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B8" s="5" t="str">
-        <f>"1/1"</f>
-        <v>1/1</v>
-      </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="8" t="e">
+        <f>"100/1"</f>
+        <v>100/1</v>
+      </c>
+      <c r="C8" s="7">
+        <v>1.69</v>
+      </c>
+      <c r="D8" s="8">
         <f>((C8)*(H8)*(I8))/(G8*1)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E8" s="8" t="e">
+        <v>138207.39286882564</v>
+      </c>
+      <c r="E8" s="8">
         <f>D8/10000</f>
-        <v>#DIV/0!</v>
+        <v>13.820739286882564</v>
       </c>
       <c r="G8" s="9">
-        <f>digestion_page!B24</f>
-        <v>0</v>
+        <f>digestion_page!B22</f>
+        <v>0.30570000000000003</v>
       </c>
       <c r="H8" s="9">
-        <f>digestion_page!C24</f>
+        <f>digestion_page!C22</f>
         <v>250</v>
       </c>
       <c r="I8" s="9">
         <f>(LEFT(B8,FIND("/",B8)-1)/RIGHT(B8,LEN(B8)-FIND("/", B8)))</f>
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" s="18"/>
-      <c r="C10" s="11" t="e">
+      <c r="C10" s="11">
         <f>AVERAGE(D7:D8)</f>
-        <v>#DIV/0!</v>
+        <v>137937.19268726392</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="18" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B11" s="18"/>
-      <c r="C11" s="12" t="e">
+      <c r="C11" s="12">
         <f>AVERAGE(E7:E8)</f>
-        <v>#DIV/0!</v>
+        <v>13.793719268726392</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="18" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B12" s="18"/>
-      <c r="C12" s="3"/>
+      <c r="C12" s="3">
+        <v>1.399</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="12" t="e">
+      <c r="A13" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="21"/>
+      <c r="C13" s="22">
         <f>AVERAGE(E7:E8)*(C12)</f>
-        <v>#DIV/0!</v>
+        <v>19.297413256948222</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B14" s="18"/>
       <c r="C14" s="19"/>
@@ -1687,7 +1471,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B16" s="10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C16" s="20"/>
       <c r="D16" s="20"/>
@@ -1726,8 +1510,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:A23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1736,67 +1520,67 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
close to finish product
</commit_message>
<xml_diff>
--- a/dist/master_workbook.xlsx
+++ b/dist/master_workbook.xlsx
@@ -8,15 +8,16 @@
   </bookViews>
   <sheets>
     <sheet name="digestion_page" sheetId="1" r:id="rId1"/>
-    <sheet name="2" sheetId="2" r:id="rId2"/>
-    <sheet name="formula_page" sheetId="3" r:id="rId3"/>
+    <sheet name="200126511" sheetId="2" r:id="rId2"/>
+    <sheet name="200126512" sheetId="3" r:id="rId3"/>
+    <sheet name="formula_page" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="55">
   <si>
     <t>Date:</t>
   </si>
@@ -75,10 +76,16 @@
     <t>volume (mL)</t>
   </si>
   <si>
-    <t>2_1</t>
-  </si>
-  <si>
-    <t>2_2</t>
+    <t>200126511_1</t>
+  </si>
+  <si>
+    <t>200126511_2</t>
+  </si>
+  <si>
+    <t>200126512_1</t>
+  </si>
+  <si>
+    <t>200126512_2</t>
   </si>
   <si>
     <t>Ca ICP analysis</t>
@@ -604,7 +611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -777,6 +784,20 @@
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="6"/>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="8"/>
+      <c r="C19" s="6"/>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="8"/>
+      <c r="C20" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -822,25 +843,25 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B5" s="3"/>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -905,7 +926,7 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="13">
@@ -915,7 +936,7 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="14">
@@ -925,14 +946,14 @@
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="12" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="3"/>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="14">
@@ -942,11 +963,11 @@
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="12" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="15" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D14" s="15"/>
       <c r="E14" s="15"/>
@@ -954,25 +975,25 @@
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B16" s="3"/>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1037,7 +1058,7 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="13">
@@ -1047,7 +1068,7 @@
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="12" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="14">
@@ -1057,14 +1078,14 @@
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="12" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="3"/>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="12" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B24" s="12"/>
       <c r="C24" s="14">
@@ -1074,7 +1095,7 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="12" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="15"/>
@@ -1084,7 +1105,7 @@
     </row>
     <row r="27" spans="1:9">
       <c r="B27" s="12" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
@@ -1137,6 +1158,349 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I29"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="3"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="10">
+        <f>((C7)*(H7)*(I7))/(G7*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="10">
+        <f>D7/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="11">
+        <f>digestion_page!B19</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="11">
+        <f>digestion_page!C19</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="11">
+        <f>(LEFT(B7,FIND("/",B7)-1)/RIGHT(B7,LEN(B7)-FIND("/", B7)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="10">
+        <f>((C8)*(H8)*(I8))/(G8*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="10">
+        <f>D8/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="11">
+        <f>digestion_page!B20</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="11">
+        <f>digestion_page!C20</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="11">
+        <f>(LEFT(B8,FIND("/",B8)-1)/RIGHT(B8,LEN(B8)-FIND("/", B8)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="12"/>
+      <c r="C10" s="13">
+        <f>AVERAGE(D7:D8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="12"/>
+      <c r="C11" s="14">
+        <f>AVERAGE(E7:E8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="12"/>
+      <c r="C12" s="3"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="12"/>
+      <c r="C13" s="14">
+        <f>AVERAGE(E7:E8)*(C12)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="12"/>
+      <c r="C14" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="3"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C18" s="9"/>
+      <c r="D18" s="10">
+        <f>((C18)*(H18)*(I18))/(G18*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="10">
+        <f>D18/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="11">
+        <f>digestion_page!B19</f>
+        <v>0</v>
+      </c>
+      <c r="H18" s="11">
+        <f>digestion_page!C19</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="11">
+        <f>(LEFT(B18,FIND("/",B18)-1)/RIGHT(B18,LEN(B18)-FIND("/", B18)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="6">
+        <f>"1/1"</f>
+        <v>0</v>
+      </c>
+      <c r="C19" s="9"/>
+      <c r="D19" s="10">
+        <f>((C19)*(H19)*(I19))/(G19*1)</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="10">
+        <f>D19/10000</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="11">
+        <f>digestion_page!B20</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="11">
+        <f>digestion_page!C20</f>
+        <v>0</v>
+      </c>
+      <c r="I19" s="11">
+        <f>(LEFT(B19,FIND("/",B19)-1)/RIGHT(B19,LEN(B19)-FIND("/", B19)))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="12"/>
+      <c r="C21" s="13">
+        <f>AVERAGE(D18:D19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B22" s="12"/>
+      <c r="C22" s="14">
+        <f>AVERAGE(E18:E19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="12"/>
+      <c r="C23" s="3"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24" s="12"/>
+      <c r="C24" s="14">
+        <f>AVERAGE(E18:E19)*(C23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="12"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="B27" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="C27:F29"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C14:F14">
+    <cfRule type="containsBlanks" dxfId="0" priority="1">
+      <formula>LEN(TRIM(C14))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C25:F25">
+    <cfRule type="containsBlanks" dxfId="0" priority="2">
+      <formula>LEN(TRIM(C25))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1145,67 +1509,67 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="17" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="17" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="17" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="17" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="17" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="17" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="17" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="17" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="17" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="17" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="17" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" s="17" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>